<commit_message>
Backend Review functionality for Sprint 2 updates from Ali
</commit_message>
<xml_diff>
--- a/src/data/campus_locations.xlsx
+++ b/src/data/campus_locations.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\CP317\Group Assignment\HawkMaps\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A41FA82-3394-44EB-8969-E11FA777242E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B85D54-1CF7-4A1A-92B7-EAFEFAB981A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="83">
   <si>
     <t>Campus Locations &amp; Coordinates (Condensed Format)</t>
   </si>
@@ -106,15 +106,9 @@
     <t>8:30 am – 11:00 pm, Mon - Thurs.8:30 am – 5:00 pm, Fri.11:00 am – 5:00 pm, Sun</t>
   </si>
   <si>
-    <t>University College</t>
-  </si>
-  <si>
     <t>8:30 am – 4:30 pm, Mon - Fri</t>
   </si>
   <si>
-    <t>Department of Co-op and Career</t>
-  </si>
-  <si>
     <t>192 King Street N</t>
   </si>
   <si>
@@ -124,12 +118,6 @@
     <t>Dining Hall</t>
   </si>
   <si>
-    <t>Welcome Centre (main entrance)</t>
-  </si>
-  <si>
-    <t>Regina St. Building</t>
-  </si>
-  <si>
     <t>202 Regina Street</t>
   </si>
   <si>
@@ -139,9 +127,6 @@
     <t>12 Lodge Street</t>
   </si>
   <si>
-    <t>232 King Street North</t>
-  </si>
-  <si>
     <t>232 King Street N</t>
   </si>
   <si>
@@ -172,9 +157,6 @@
     <t>7:30 am – 7:00 pm, Mon - Thu.7:30 am – 5:00 pm, Fri.9:00 am – 5:00 pm, Sat - Sun</t>
   </si>
   <si>
-    <t>Torque (Dining Hall)</t>
-  </si>
-  <si>
     <t>Chamberlain Music</t>
   </si>
   <si>
@@ -269,6 +251,27 @@
   </si>
   <si>
     <t>Study</t>
+  </si>
+  <si>
+    <t>Martin Luther University College</t>
+  </si>
+  <si>
+    <t>Co-op and Career Centre</t>
+  </si>
+  <si>
+    <t>MacDonald House (main entrance)</t>
+  </si>
+  <si>
+    <t>Regina Administration Building</t>
+  </si>
+  <si>
+    <t>WLU Campus Police</t>
+  </si>
+  <si>
+    <t>Community and Workplace Partnerships</t>
+  </si>
+  <si>
+    <t>Fresh Food Company (Dining Hall)</t>
   </si>
 </sst>
 </file>
@@ -278,7 +281,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -301,6 +304,22 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -335,7 +354,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -358,11 +377,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -387,6 +419,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -726,18 +770,18 @@
         <v>5</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3">
-        <v>43.47345</v>
-      </c>
-      <c r="C4" s="3">
-        <v>-80.527519999999996</v>
+      <c r="B4" s="12">
+        <v>43.473805302175101</v>
+      </c>
+      <c r="C4" s="9">
+        <v>-80.529750608316206</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>7</v>
@@ -754,10 +798,10 @@
         <v>9</v>
       </c>
       <c r="B5" s="6">
-        <v>43.47345</v>
+        <v>43.472727658618602</v>
       </c>
       <c r="C5" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.526467892662296</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
@@ -774,10 +818,10 @@
         <v>10</v>
       </c>
       <c r="B6" s="3">
-        <v>43.472740000000002</v>
+        <v>43.4745253826311</v>
       </c>
       <c r="C6" s="3">
-        <v>-80.525350000000003</v>
+        <v>-80.520921870892394</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>11</v>
@@ -794,10 +838,10 @@
         <v>13</v>
       </c>
       <c r="B7" s="6">
-        <v>43.47345</v>
+        <v>43.473898674046602</v>
       </c>
       <c r="C7" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.529451820604805</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>7</v>
@@ -806,7 +850,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -814,10 +858,10 @@
         <v>14</v>
       </c>
       <c r="B8" s="3">
-        <v>43.47345</v>
+        <v>43.4733080827748</v>
       </c>
       <c r="C8" s="3">
-        <v>-80.527519999999996</v>
+        <v>-80.529424501731697</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>7</v>
@@ -834,10 +878,10 @@
         <v>15</v>
       </c>
       <c r="B9" s="6">
-        <v>43.47345</v>
+        <v>43.473705868546503</v>
       </c>
       <c r="C9" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.530550065926704</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>7</v>
@@ -854,10 +898,10 @@
         <v>16</v>
       </c>
       <c r="B10" s="3">
-        <v>43.47345</v>
+        <v>43.474229716674301</v>
       </c>
       <c r="C10" s="3">
-        <v>-80.527519999999996</v>
+        <v>-80.527858651926294</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>7</v>
@@ -866,7 +910,7 @@
         <v>8</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -874,10 +918,10 @@
         <v>17</v>
       </c>
       <c r="B11" s="6">
-        <v>43.47345</v>
+        <v>43.474489565304197</v>
       </c>
       <c r="C11" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.528228796764296</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>7</v>
@@ -886,7 +930,7 @@
         <v>12</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -894,10 +938,10 @@
         <v>18</v>
       </c>
       <c r="B12" s="3">
-        <v>43.475119999999997</v>
+        <v>43.475028756209603</v>
       </c>
       <c r="C12" s="3">
-        <v>-80.529539999999997</v>
+        <v>-80.529465298489896</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>19</v>
@@ -914,10 +958,10 @@
         <v>20</v>
       </c>
       <c r="B13" s="6">
-        <v>43.476410000000001</v>
+        <v>43.477635581942501</v>
       </c>
       <c r="C13" s="6">
-        <v>-80.527029999999996</v>
+        <v>-80.531500785618206</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>21</v>
@@ -934,10 +978,10 @@
         <v>22</v>
       </c>
       <c r="B14" s="3">
-        <v>43.47345</v>
+        <v>43.4732827352044</v>
       </c>
       <c r="C14" s="3">
-        <v>-80.527519999999996</v>
+        <v>-80.530321785667198</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>7</v>
@@ -954,10 +998,10 @@
         <v>23</v>
       </c>
       <c r="B15" s="6">
-        <v>43.47345</v>
+        <v>43.473471831975402</v>
       </c>
       <c r="C15" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.524923838104797</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>7</v>
@@ -974,10 +1018,10 @@
         <v>24</v>
       </c>
       <c r="B16" s="3">
-        <v>43.47345</v>
+        <v>43.473064557408001</v>
       </c>
       <c r="C16" s="3">
-        <v>-80.527519999999996</v>
+        <v>-80.525986427008704</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>7</v>
@@ -986,7 +1030,7 @@
         <v>8</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -994,10 +1038,10 @@
         <v>25</v>
       </c>
       <c r="B17" s="6">
-        <v>43.47345</v>
+        <v>43.472952595933897</v>
       </c>
       <c r="C17" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.5298989716146</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>7</v>
@@ -1006,24 +1050,24 @@
         <v>26</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>27</v>
+        <v>76</v>
       </c>
       <c r="B18" s="3">
-        <v>43.47345</v>
+        <v>43.472026291626101</v>
       </c>
       <c r="C18" s="3">
-        <v>-80.527519999999996</v>
+        <v>-80.528725553670299</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>1</v>
@@ -1031,19 +1075,19 @@
     </row>
     <row r="19" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="6">
+        <v>43.473943413659299</v>
+      </c>
+      <c r="C19" s="6">
+        <v>-80.524135288415295</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="B19" s="6">
-        <v>43.474110000000003</v>
-      </c>
-      <c r="C19" s="6">
-        <v>-80.522819999999996</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>31</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>1</v>
@@ -1051,13 +1095,13 @@
     </row>
     <row r="20" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B20" s="3">
-        <v>43.47345</v>
+        <v>43.474421388064201</v>
       </c>
       <c r="C20" s="3">
-        <v>-80.527519999999996</v>
+        <v>-80.528695093872798</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>7</v>
@@ -1066,24 +1110,24 @@
         <v>8</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="B21" s="6">
-        <v>43.47345</v>
+        <v>43.473752067616402</v>
       </c>
       <c r="C21" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.527991639021806</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>1</v>
@@ -1091,59 +1135,59 @@
     </row>
     <row r="22" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" s="3">
+        <v>43.474696656654899</v>
+      </c>
+      <c r="C22" s="3">
+        <v>-80.5226718993313</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="6">
+        <v>43.473980743854803</v>
+      </c>
+      <c r="C23" s="6">
+        <v>-80.523576832013902</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="3">
+        <v>43.475379071181997</v>
+      </c>
+      <c r="C24" s="3">
+        <v>-80.524446125988803</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="3">
-        <v>43.472580000000001</v>
-      </c>
-      <c r="C22" s="3">
-        <v>-80.52422</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="E24" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B23" s="6">
-        <v>43.471649999999997</v>
-      </c>
-      <c r="C23" s="6">
-        <v>-80.525120000000001</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B24" s="3">
-        <v>43.475540000000002</v>
-      </c>
-      <c r="C24" s="3">
-        <v>-80.522229999999993</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>1</v>
@@ -1151,259 +1195,259 @@
     </row>
     <row r="25" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B25" s="6">
-        <v>43.475119999999997</v>
+        <v>43.4750324939913</v>
       </c>
       <c r="C25" s="6">
-        <v>-80.529539999999997</v>
+        <v>-80.528796298303902</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B26" s="3">
-        <v>43.473120000000002</v>
+        <v>43.473536910322601</v>
       </c>
       <c r="C26" s="3">
-        <v>-80.528239999999997</v>
+        <v>-80.528676934596106</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B27" s="6">
-        <v>43.47345</v>
+        <v>43.473643932139701</v>
       </c>
       <c r="C27" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.529140017146304</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="B28" s="3">
-        <v>43.47231</v>
+        <v>43.474315388868803</v>
       </c>
       <c r="C28" s="3">
-        <v>-80.528919999999999</v>
+        <v>-80.528655665623305</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B29" s="6">
-        <v>43.473120000000002</v>
+        <v>43.473480688269802</v>
       </c>
       <c r="C29" s="6">
-        <v>-80.528239999999997</v>
+        <v>-80.528736361520401</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B30" s="3">
-        <v>43.473120000000002</v>
+        <v>43.473394915644398</v>
       </c>
       <c r="C30" s="3">
-        <v>-80.528239999999997</v>
+        <v>-80.528582873445799</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B31" s="6">
-        <v>43.473120000000002</v>
+        <v>43.473425293463201</v>
       </c>
       <c r="C31" s="6">
-        <v>-80.528239999999997</v>
+        <v>-80.528820082288405</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B32" s="3">
-        <v>43.473120000000002</v>
+        <v>43.473484973892603</v>
       </c>
       <c r="C32" s="3">
-        <v>-80.528239999999997</v>
+        <v>-80.528788619853799</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B33" s="6">
-        <v>43.473120000000002</v>
+        <v>43.473433392684399</v>
       </c>
       <c r="C33" s="6">
-        <v>-80.528239999999997</v>
+        <v>-80.528732293465495</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B34" s="3">
-        <v>43.47345</v>
+        <v>43.472674523217499</v>
       </c>
       <c r="C34" s="3">
-        <v>-80.527519999999996</v>
+        <v>-80.526391671476901</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B35" s="6">
-        <v>43.47345</v>
+        <v>43.473195664874197</v>
       </c>
       <c r="C35" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.525516231768904</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B36" s="3">
-        <v>43.473120000000002</v>
+        <v>43.473520046064003</v>
       </c>
       <c r="C36" s="3">
-        <v>-80.528239999999997</v>
+        <v>-80.528771058239599</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>12</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B37" s="6">
-        <v>43.473820000000003</v>
+        <v>43.473387227739103</v>
       </c>
       <c r="C37" s="6">
-        <v>-80.526840000000007</v>
+        <v>-80.529436767708901</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>1</v>
@@ -1411,19 +1455,19 @@
     </row>
     <row r="38" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B38" s="3">
-        <v>43.473120000000002</v>
+        <v>43.473575452387898</v>
       </c>
       <c r="C38" s="3">
-        <v>-80.528239999999997</v>
+        <v>-80.528657486472994</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>1</v>
@@ -1431,19 +1475,19 @@
     </row>
     <row r="39" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="B39" s="6">
-        <v>43.473350000000003</v>
+        <v>43.473703851079897</v>
       </c>
       <c r="C39" s="6">
-        <v>-80.527119999999996</v>
+        <v>-80.529310228738694</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>1</v>
@@ -1451,19 +1495,19 @@
     </row>
     <row r="40" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B40" s="3">
-        <v>43.473120000000002</v>
+        <v>43.473613855449699</v>
       </c>
       <c r="C40" s="3">
-        <v>-80.528239999999997</v>
+        <v>-80.528824038492203</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>1</v>
@@ -1471,19 +1515,19 @@
     </row>
     <row r="41" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B41" s="6">
-        <v>43.47345</v>
+        <v>43.475219485099501</v>
       </c>
       <c r="C41" s="6">
-        <v>-80.527519999999996</v>
+        <v>-80.5257567223602</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>1</v>

</xml_diff>